<commit_message>
Ruteo estatico sin contar guatemala
</commit_message>
<xml_diff>
--- a/Subneteo.xlsx
+++ b/Subneteo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Bendaña\Documents\U\Redes\Proyecto Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DCF5C1E-752E-4814-9711-3F612FF01F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C57C146-AD00-4124-BF4A-94B94DEECEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="105" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{B81E0653-01D2-4AC0-8BA6-03BB38D3D29D}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B81E0653-01D2-4AC0-8BA6-03BB38D3D29D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="254">
   <si>
     <t>RED</t>
   </si>
@@ -786,6 +786,258 @@
   </si>
   <si>
     <t xml:space="preserve">SERVIDORES = </t>
+  </si>
+  <si>
+    <t>RED WAN</t>
+  </si>
+  <si>
+    <t>183.168.100.1</t>
+  </si>
+  <si>
+    <t>183.168.100.2</t>
+  </si>
+  <si>
+    <t>183.168.100.3</t>
+  </si>
+  <si>
+    <t>183.168.100.5</t>
+  </si>
+  <si>
+    <t>183.168.100.6</t>
+  </si>
+  <si>
+    <t>183.168.100.7</t>
+  </si>
+  <si>
+    <t>183.168.100.9</t>
+  </si>
+  <si>
+    <t>183.168.100.10</t>
+  </si>
+  <si>
+    <t>183.168.100.11</t>
+  </si>
+  <si>
+    <t>183.168.100.13</t>
+  </si>
+  <si>
+    <t>183.168.100.14</t>
+  </si>
+  <si>
+    <t>183.168.100.15</t>
+  </si>
+  <si>
+    <t>183.168.100.17</t>
+  </si>
+  <si>
+    <t>183.168.100.18</t>
+  </si>
+  <si>
+    <t>183.168.100.19</t>
+  </si>
+  <si>
+    <t>183.168.100.21</t>
+  </si>
+  <si>
+    <t>183.168.100.22</t>
+  </si>
+  <si>
+    <t>183.168.100.23</t>
+  </si>
+  <si>
+    <t>183.168.100.25</t>
+  </si>
+  <si>
+    <t>183.168.100.26</t>
+  </si>
+  <si>
+    <t>183.168.100.27</t>
+  </si>
+  <si>
+    <t>183.168.100.0</t>
+  </si>
+  <si>
+    <t>183.168.100.4</t>
+  </si>
+  <si>
+    <t>183.168.100.8</t>
+  </si>
+  <si>
+    <t>183.168.100.12</t>
+  </si>
+  <si>
+    <t>183.168.100.16</t>
+  </si>
+  <si>
+    <t>183.168.100.24</t>
+  </si>
+  <si>
+    <t>183.168.100.20</t>
+  </si>
+  <si>
+    <t>LUGAR</t>
+  </si>
+  <si>
+    <t>Tegucigalpa</t>
+  </si>
+  <si>
+    <t>San Pedro Sula</t>
+  </si>
+  <si>
+    <t>Guatemala</t>
+  </si>
+  <si>
+    <t>Miami</t>
+  </si>
+  <si>
+    <t>San Jose Costa Rica</t>
+  </si>
+  <si>
+    <t>Panama</t>
+  </si>
+  <si>
+    <t>Atlanta</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>183.168.100.28</t>
+  </si>
+  <si>
+    <t>183.168.100.29</t>
+  </si>
+  <si>
+    <t>183.168.100.30</t>
+  </si>
+  <si>
+    <t>183.168.100.31</t>
+  </si>
+  <si>
+    <t>Costa Rica - Panama</t>
+  </si>
+  <si>
+    <t>Panama - Costa Rica</t>
+  </si>
+  <si>
+    <t>Panama - Tegucigalpa</t>
+  </si>
+  <si>
+    <t>Panama - San Pedro Sula</t>
+  </si>
+  <si>
+    <t>Panama - Miami</t>
+  </si>
+  <si>
+    <t>Panama - Atlanta</t>
+  </si>
+  <si>
+    <t>Panama - New York</t>
+  </si>
+  <si>
+    <t>Costa Rica - Tegucigalpa</t>
+  </si>
+  <si>
+    <t>Costa Rica - San Pedro Sula</t>
+  </si>
+  <si>
+    <t>Costa Rica - Miami</t>
+  </si>
+  <si>
+    <t>Costa Rica - Atlanta</t>
+  </si>
+  <si>
+    <t>Costa Rica - New York</t>
+  </si>
+  <si>
+    <t>Tegucigalpa - Panama</t>
+  </si>
+  <si>
+    <t>Tegucigalpa - Costa Rica</t>
+  </si>
+  <si>
+    <t>Tegucigalpa - San Pedro Sula</t>
+  </si>
+  <si>
+    <t>Tegucigalpa - Miami</t>
+  </si>
+  <si>
+    <t>Tegucigalpa - Atlanta</t>
+  </si>
+  <si>
+    <t>Tegucigalpa - New York</t>
+  </si>
+  <si>
+    <t>San Pedro Sula - Panama</t>
+  </si>
+  <si>
+    <t>Miami - Panama</t>
+  </si>
+  <si>
+    <t>Miami - Costa Rica</t>
+  </si>
+  <si>
+    <t>Miami - Tegucigalpa</t>
+  </si>
+  <si>
+    <t>Miami - San Pedro Sula</t>
+  </si>
+  <si>
+    <t>Miami - Atlanta</t>
+  </si>
+  <si>
+    <t>Miami - New York</t>
+  </si>
+  <si>
+    <t>San Pedro Sula - Costa Rica</t>
+  </si>
+  <si>
+    <t>San Pedro Sula - Tegucigalpa</t>
+  </si>
+  <si>
+    <t>San Pedro Sula - Miami</t>
+  </si>
+  <si>
+    <t>San Pedro Sula - Atlanta</t>
+  </si>
+  <si>
+    <t>San Pedro Sula - New York</t>
+  </si>
+  <si>
+    <t>Atlanta - Panama</t>
+  </si>
+  <si>
+    <t>Atlanta - Costa Rica</t>
+  </si>
+  <si>
+    <t>Atlanta - Tegucigalpa</t>
+  </si>
+  <si>
+    <t>Atlanta - San Pedro Sula</t>
+  </si>
+  <si>
+    <t>Atlanta - Miami</t>
+  </si>
+  <si>
+    <t>Atlanta - New York</t>
+  </si>
+  <si>
+    <t>New York - Panama</t>
+  </si>
+  <si>
+    <t>New York - Costa Rica</t>
+  </si>
+  <si>
+    <t>New York - Tegucigalpa</t>
+  </si>
+  <si>
+    <t>New York - San Pedro Sula</t>
+  </si>
+  <si>
+    <t>New York - Miami</t>
+  </si>
+  <si>
+    <t>New York - Atlanta</t>
   </si>
 </sst>
 </file>
@@ -821,7 +1073,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -849,6 +1101,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -917,19 +1181,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -948,12 +1206,41 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF00FF00"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1198,7 +1485,7 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>295275</xdr:colOff>
       <xdr:row>54</xdr:row>
-      <xdr:rowOff>88589</xdr:rowOff>
+      <xdr:rowOff>43765</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1355,6 +1642,50 @@
         <a:xfrm>
           <a:off x="0" y="7597589"/>
           <a:ext cx="5670176" cy="976760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>180976</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>60034</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD3711C9-58FE-9423-E20F-EDF6C368BD4D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="10896601"/>
+          <a:ext cx="5648325" cy="2165058"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1683,31 +2014,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{158608C6-5E75-45EA-AC37-234E2DEA60DD}">
-  <dimension ref="I1:U43"/>
+  <dimension ref="I1:U66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="9" max="9" width="19.5703125" customWidth="1"/>
-    <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="17.5703125" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="16.5703125" customWidth="1"/>
-    <col min="15" max="15" width="8" customWidth="1"/>
+    <col min="9" max="9" width="21.140625" customWidth="1"/>
+    <col min="10" max="10" width="23.28515625" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" customWidth="1"/>
+    <col min="15" max="15" width="24.140625" customWidth="1"/>
+    <col min="16" max="16" width="5.85546875" customWidth="1"/>
     <col min="17" max="17" width="16.28515625" customWidth="1"/>
     <col min="18" max="18" width="26" customWidth="1"/>
     <col min="21" max="21" width="35.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
     </row>
     <row r="2" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I2" s="1" t="s">
@@ -1847,15 +2179,15 @@
       </c>
     </row>
     <row r="7" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
     </row>
     <row r="8" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I8" s="4" t="s">
@@ -1995,15 +2327,15 @@
       </c>
     </row>
     <row r="13" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I13" s="6" t="s">
+      <c r="I13" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
     </row>
     <row r="14" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I14" s="1" t="s">
@@ -2105,15 +2437,15 @@
       </c>
     </row>
     <row r="18" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
     </row>
     <row r="19" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I19" s="4" t="s">
@@ -2253,15 +2585,15 @@
       </c>
     </row>
     <row r="24" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I24" s="6" t="s">
+      <c r="I24" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
-      <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="6"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
     </row>
     <row r="25" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I25" s="1" t="s">
@@ -2363,15 +2695,15 @@
       </c>
     </row>
     <row r="29" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I29" s="11" t="s">
+      <c r="I29" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
-      <c r="L29" s="12"/>
-      <c r="M29" s="12"/>
-      <c r="N29" s="12"/>
-      <c r="O29" s="13"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="11"/>
     </row>
     <row r="30" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I30" s="4" t="s">
@@ -2473,15 +2805,15 @@
       </c>
     </row>
     <row r="34" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I34" s="8" t="s">
+      <c r="I34" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="J34" s="9"/>
-      <c r="K34" s="9"/>
-      <c r="L34" s="9"/>
-      <c r="M34" s="9"/>
-      <c r="N34" s="9"/>
-      <c r="O34" s="10"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="7"/>
+      <c r="L34" s="7"/>
+      <c r="M34" s="7"/>
+      <c r="N34" s="7"/>
+      <c r="O34" s="8"/>
     </row>
     <row r="35" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I35" s="1" t="s">
@@ -2583,15 +2915,15 @@
       </c>
     </row>
     <row r="39" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I39" s="11" t="s">
+      <c r="I39" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="J39" s="12"/>
-      <c r="K39" s="12"/>
-      <c r="L39" s="12"/>
-      <c r="M39" s="12"/>
-      <c r="N39" s="12"/>
-      <c r="O39" s="13"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="10"/>
+      <c r="N39" s="10"/>
+      <c r="O39" s="11"/>
     </row>
     <row r="40" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I40" s="4" t="s">
@@ -2730,8 +3062,377 @@
         <v>149</v>
       </c>
     </row>
+    <row r="46" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="I46" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="J46" s="16"/>
+      <c r="K46" s="16"/>
+      <c r="L46" s="16"/>
+      <c r="M46" s="16"/>
+      <c r="N46" s="16"/>
+      <c r="O46" s="16"/>
+    </row>
+    <row r="47" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="I47" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="J47" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="K47" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="L47" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="M47" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="N47" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="O47" s="14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="I48" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O48" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="49" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I49" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="M49" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O49" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="50" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I50" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O50" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="51" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I51" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O51" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="52" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I52" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="M52" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="N52" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O52" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="53" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I53" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O53" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="54" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I54" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O54" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="55" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I55" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="M55" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O55" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="56" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="R56" s="18"/>
+    </row>
+    <row r="58" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I58" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="J58" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="K58" s="21" t="s">
+        <v>224</v>
+      </c>
+      <c r="L58" s="21" t="s">
+        <v>230</v>
+      </c>
+      <c r="M58" s="21" t="s">
+        <v>231</v>
+      </c>
+      <c r="N58" s="21" t="s">
+        <v>242</v>
+      </c>
+      <c r="O58" s="21" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="59" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I59" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="J59" s="21" t="s">
+        <v>219</v>
+      </c>
+      <c r="K59" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="L59" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="M59" s="21" t="s">
+        <v>232</v>
+      </c>
+      <c r="N59" s="21" t="s">
+        <v>243</v>
+      </c>
+      <c r="O59" s="21" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="60" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I60" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="J60" s="21" t="s">
+        <v>220</v>
+      </c>
+      <c r="K60" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="L60" s="21" t="s">
+        <v>238</v>
+      </c>
+      <c r="M60" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="N60" s="21" t="s">
+        <v>244</v>
+      </c>
+      <c r="O60" s="21" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="61" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I61" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="J61" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="K61" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="L61" s="21" t="s">
+        <v>239</v>
+      </c>
+      <c r="M61" s="21" t="s">
+        <v>234</v>
+      </c>
+      <c r="N61" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="O61" s="21" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="62" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I62" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="J62" s="21" t="s">
+        <v>222</v>
+      </c>
+      <c r="K62" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="L62" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="M62" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="N62" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="O62" s="21" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="63" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I63" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="J63" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="K63" s="21" t="s">
+        <v>229</v>
+      </c>
+      <c r="L63" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="M63" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="N63" s="21" t="s">
+        <v>247</v>
+      </c>
+      <c r="O63" s="21" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="64" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I64" s="19"/>
+    </row>
+    <row r="65" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I65" s="19"/>
+    </row>
+    <row r="66" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I66" s="19"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="I46:O46"/>
     <mergeCell ref="I34:O34"/>
     <mergeCell ref="I39:O39"/>
     <mergeCell ref="I29:O29"/>

</xml_diff>

<commit_message>
Segun ya esta terminado
</commit_message>
<xml_diff>
--- a/Subneteo.xlsx
+++ b/Subneteo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Bendaña\Documents\U\Redes\Proyecto Final - Copy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F2E360-9926-4005-A19C-CF6AB8C8A612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9E8518-DA50-4371-AEE8-A40D9B7A608C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B81E0653-01D2-4AC0-8BA6-03BB38D3D29D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="292">
   <si>
     <t>RED</t>
   </si>
@@ -875,33 +875,6 @@
     <t>183.168.100.20</t>
   </si>
   <si>
-    <t>LUGAR</t>
-  </si>
-  <si>
-    <t>Tegucigalpa</t>
-  </si>
-  <si>
-    <t>San Pedro Sula</t>
-  </si>
-  <si>
-    <t>Guatemala</t>
-  </si>
-  <si>
-    <t>Miami</t>
-  </si>
-  <si>
-    <t>San Jose Costa Rica</t>
-  </si>
-  <si>
-    <t>Panama</t>
-  </si>
-  <si>
-    <t>Atlanta</t>
-  </si>
-  <si>
-    <t>New York</t>
-  </si>
-  <si>
     <t>183.168.100.28</t>
   </si>
   <si>
@@ -1040,19 +1013,145 @@
     <t>New York - Atlanta</t>
   </si>
   <si>
-    <t>Extra</t>
-  </si>
-  <si>
-    <t>183.168.100.32</t>
-  </si>
-  <si>
-    <t>183.168.100.33</t>
-  </si>
-  <si>
-    <t>183.168.100.34</t>
-  </si>
-  <si>
-    <t>183.168.100.35</t>
+    <t>DISPONIBLES</t>
+  </si>
+  <si>
+    <t>UTILIZADOS</t>
+  </si>
+  <si>
+    <t>NIVEL</t>
+  </si>
+  <si>
+    <t>10.10.10.5 - 10.10.10.126</t>
+  </si>
+  <si>
+    <t>10.10.10.133 - 10.10.10.190</t>
+  </si>
+  <si>
+    <t>10.10.10.197 - 10.10.10.254</t>
+  </si>
+  <si>
+    <t>10.10.10.1 - 10.10.10.4</t>
+  </si>
+  <si>
+    <t>11.11.10.1 - 11.11.10.4</t>
+  </si>
+  <si>
+    <t>10.10.10.129 - 10.10.10.132</t>
+  </si>
+  <si>
+    <t>10.10.10.193 - 10.10.10.196</t>
+  </si>
+  <si>
+    <t>11.11.10.65 - 11.11.10.70</t>
+  </si>
+  <si>
+    <t>11.11.10.97 - 11.11.10.101</t>
+  </si>
+  <si>
+    <t>11.11.10.5 - 11.11.10.62</t>
+  </si>
+  <si>
+    <t>11.11.10.71 - 11.11.10.94</t>
+  </si>
+  <si>
+    <t>11.11.10.102 - 11.11.10.110</t>
+  </si>
+  <si>
+    <t>14.14.14.1 - 14.14.14.5</t>
+  </si>
+  <si>
+    <t>14.14.14.33 - 14.14.14.38</t>
+  </si>
+  <si>
+    <t>14.14.14.39 - 14.14.14.62</t>
+  </si>
+  <si>
+    <t>14.14.14.6 - 14.14.14.30</t>
+  </si>
+  <si>
+    <t>12.12.12.1 - 12.12.12.5</t>
+  </si>
+  <si>
+    <t>12.12.12.6 - 12.12.12.126</t>
+  </si>
+  <si>
+    <t>12.12.12.129 - 12.12.12.134</t>
+  </si>
+  <si>
+    <t>12.12.12.135 - 12.12.12.190</t>
+  </si>
+  <si>
+    <t>12.12.12.193  - 12.12.12.194</t>
+  </si>
+  <si>
+    <t>NINGUNO</t>
+  </si>
+  <si>
+    <t>15.15.15.1 - 15.15.15.5</t>
+  </si>
+  <si>
+    <t>15.15.15.6 - 15.15.15.30</t>
+  </si>
+  <si>
+    <t>15.15.15.33 - 15.15.15.38</t>
+  </si>
+  <si>
+    <t>15.15.15.39 - 15.15.15.62</t>
+  </si>
+  <si>
+    <t>13.13.13.1 - 13.13.13.4</t>
+  </si>
+  <si>
+    <t>13.13.13.5 - 13.13.13.30</t>
+  </si>
+  <si>
+    <t>13.13.13.33 - 13.13.13.38</t>
+  </si>
+  <si>
+    <t>13.13.13.39 - 13.13.13.62</t>
+  </si>
+  <si>
+    <t>8.8.8.1 - 8.8.8.3</t>
+  </si>
+  <si>
+    <t>8.8.8.4 - 8.8.8.6</t>
+  </si>
+  <si>
+    <t>8.8.8.9 - 8.8.8.12</t>
+  </si>
+  <si>
+    <t>8.8.8.13 - 8.8.8.14</t>
+  </si>
+  <si>
+    <t>9.9.9.1 - 9.9.9.4</t>
+  </si>
+  <si>
+    <t>9.9.9.5 - 9.9.9.126</t>
+  </si>
+  <si>
+    <t>9.9.9.129 - 9.9.9.134</t>
+  </si>
+  <si>
+    <t>9.9.9.135 - 9.9.9.190</t>
+  </si>
+  <si>
+    <t>9.9.9.193 - 9.9.9.197</t>
+  </si>
+  <si>
+    <t>9.9.9.198 - 9.9.9.254</t>
+  </si>
+  <si>
+    <t>OFICINAS</t>
+  </si>
+  <si>
+    <t>Guatemala - Tegucigalpa</t>
+  </si>
+  <si>
+    <t>Atlanta - Guatemala</t>
+  </si>
+  <si>
+    <t>NUMERO DE SUBRED</t>
   </si>
 </sst>
 </file>
@@ -1238,10 +1337,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2028,7 +2125,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{158608C6-5E75-45EA-AC37-234E2DEA60DD}">
-  <dimension ref="I1:U66"/>
+  <dimension ref="I1:Y66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="21.140625" customWidth="1"/>
@@ -2038,26 +2135,32 @@
     <col min="13" max="13" width="20.140625" customWidth="1"/>
     <col min="14" max="14" width="20.7109375" customWidth="1"/>
     <col min="15" max="15" width="24.140625" customWidth="1"/>
-    <col min="16" max="16" width="5.85546875" customWidth="1"/>
-    <col min="17" max="17" width="16.28515625" customWidth="1"/>
-    <col min="18" max="18" width="26" customWidth="1"/>
-    <col min="21" max="21" width="35.140625" customWidth="1"/>
+    <col min="16" max="16" width="24" customWidth="1"/>
+    <col min="17" max="17" width="28.5703125" customWidth="1"/>
+    <col min="18" max="18" width="31.42578125" customWidth="1"/>
+    <col min="21" max="21" width="23.85546875" customWidth="1"/>
+    <col min="22" max="22" width="30.42578125" customWidth="1"/>
+    <col min="25" max="25" width="35.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I1" s="18" t="s">
+    <row r="1" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="I1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-    </row>
-    <row r="2" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="14"/>
+    </row>
+    <row r="2" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I2" s="1" t="s">
-        <v>36</v>
+        <v>291</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>0</v>
@@ -2077,10 +2180,22 @@
       <c r="O2" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I3" s="2" t="s">
-        <v>37</v>
+      <c r="P2" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="3" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I3" s="7">
+        <v>1</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>7</v>
@@ -2100,25 +2215,37 @@
       <c r="O3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="P3" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="S3" s="2">
+        <v>1</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="V3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="W3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="X3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="Y3" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I4" s="2" t="s">
-        <v>38</v>
+    <row r="4" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I4" s="7">
+        <v>2</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>24</v>
@@ -2138,25 +2265,37 @@
       <c r="O4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="P4" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S4" s="2">
+        <v>2</v>
+      </c>
+      <c r="U4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="V4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="S4" s="3" t="s">
+      <c r="W4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="T4" s="3" t="s">
+      <c r="X4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="U4" s="3" t="s">
+      <c r="Y4" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I5" s="2" t="s">
-        <v>39</v>
+    <row r="5" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I5" s="7">
+        <v>3</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>31</v>
@@ -2176,36 +2315,52 @@
       <c r="O5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="P5" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="S5" s="2">
+        <v>1</v>
+      </c>
+      <c r="U5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="R5" s="1" t="s">
+      <c r="V5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S5" s="3" t="s">
+      <c r="W5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="T5" s="3" t="s">
+      <c r="X5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="U5" s="3" t="s">
+      <c r="Y5" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I7" s="19" t="s">
+    <row r="7" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="I7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-    </row>
-    <row r="8" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="17"/>
+    </row>
+    <row r="8" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I8" s="4" t="s">
-        <v>36</v>
+        <v>291</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>0</v>
@@ -2225,10 +2380,22 @@
       <c r="O8" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I9" s="2" t="s">
-        <v>41</v>
+      <c r="P8" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="R8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="S8" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="9" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I9" s="7">
+        <v>1</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>43</v>
@@ -2248,25 +2415,37 @@
       <c r="O9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q9" s="4" t="s">
+      <c r="P9" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S9" s="2">
+        <v>1</v>
+      </c>
+      <c r="U9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="R9" s="4" t="s">
+      <c r="V9" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="S9" s="5" t="s">
+      <c r="W9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="T9" s="5" t="s">
+      <c r="X9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="U9" s="5" t="s">
+      <c r="Y9" s="5" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I10" s="2" t="s">
-        <v>38</v>
+    <row r="10" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I10" s="7">
+        <v>2</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>53</v>
@@ -2286,25 +2465,37 @@
       <c r="O10" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q10" s="4" t="s">
+      <c r="P10" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="R10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S10" s="2">
+        <v>2</v>
+      </c>
+      <c r="U10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="R10" s="4" t="s">
+      <c r="V10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="S10" s="5" t="s">
+      <c r="W10" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="T10" s="5" t="s">
+      <c r="X10" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="U10" s="5" t="s">
+      <c r="Y10" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I11" s="2" t="s">
-        <v>42</v>
+    <row r="11" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I11" s="7">
+        <v>3</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>62</v>
@@ -2324,23 +2515,35 @@
       <c r="O11" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="Q11" s="4" t="s">
+      <c r="P11" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S11" s="2">
+        <v>1</v>
+      </c>
+      <c r="U11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="R11" s="4" t="s">
+      <c r="V11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="S11" s="5" t="s">
+      <c r="W11" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="T11" s="5" t="s">
+      <c r="X11" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="U11" s="5" t="s">
+      <c r="Y11" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="13" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
       <c r="I13" s="18" t="s">
         <v>69</v>
       </c>
@@ -2350,10 +2553,14 @@
       <c r="M13" s="18"/>
       <c r="N13" s="18"/>
       <c r="O13" s="18"/>
-    </row>
-    <row r="14" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="P13" s="18"/>
+      <c r="Q13" s="18"/>
+      <c r="R13" s="18"/>
+      <c r="S13" s="18"/>
+    </row>
+    <row r="14" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I14" s="1" t="s">
-        <v>36</v>
+        <v>291</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>0</v>
@@ -2373,10 +2580,22 @@
       <c r="O14" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="15" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I15" s="2" t="s">
-        <v>70</v>
+      <c r="P14" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S14" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="15" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I15" s="7">
+        <v>1</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>72</v>
@@ -2396,25 +2615,37 @@
       <c r="O15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q15" s="1" t="s">
+      <c r="P15" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="S15" s="2">
+        <v>1</v>
+      </c>
+      <c r="U15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="R15" s="1" t="s">
+      <c r="V15" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="S15" s="3" t="s">
+      <c r="W15" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="T15" s="3" t="s">
+      <c r="X15" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="U15" s="3" t="s">
+      <c r="Y15" s="3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I16" s="2" t="s">
-        <v>71</v>
+    <row r="16" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I16" s="7">
+        <v>2</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>78</v>
@@ -2434,36 +2665,65 @@
       <c r="O16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q16" s="1" t="s">
+      <c r="P16" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S16" s="2">
+        <v>2</v>
+      </c>
+      <c r="U16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="R16" s="1" t="s">
+      <c r="V16" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="S16" s="3" t="s">
+      <c r="W16" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="T16" s="3" t="s">
+      <c r="X16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="U16" s="3" t="s">
+      <c r="Y16" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="18" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I18" s="19" t="s">
+    <row r="17" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="19"/>
+      <c r="O17" s="19"/>
+      <c r="P17" s="19"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="19"/>
+      <c r="S17" s="19"/>
+    </row>
+    <row r="18" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="I18" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="19"/>
-    </row>
-    <row r="19" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="17"/>
+    </row>
+    <row r="19" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I19" s="4" t="s">
-        <v>36</v>
+        <v>291</v>
       </c>
       <c r="J19" s="4" t="s">
         <v>0</v>
@@ -2483,10 +2743,22 @@
       <c r="O19" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="20" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I20" s="2" t="s">
-        <v>70</v>
+      <c r="P19" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q19" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="R19" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="S19" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="20" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I20" s="7">
+        <v>1</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>85</v>
@@ -2506,25 +2778,37 @@
       <c r="O20" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Q20" s="4" t="s">
+      <c r="P20" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="Q20" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="R20" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="S20" s="2">
+        <v>1</v>
+      </c>
+      <c r="U20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="R20" s="4" t="s">
+      <c r="V20" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="S20" s="5" t="s">
+      <c r="W20" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="T20" s="5" t="s">
+      <c r="X20" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="U20" s="5" t="s">
+      <c r="Y20" s="5" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I21" s="2" t="s">
-        <v>84</v>
+    <row r="21" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I21" s="7">
+        <v>2</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>95</v>
@@ -2544,25 +2828,37 @@
       <c r="O21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q21" s="4" t="s">
+      <c r="P21" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q21" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="R21" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="S21" s="2">
+        <v>2</v>
+      </c>
+      <c r="U21" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="R21" s="4" t="s">
+      <c r="V21" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="S21" s="5" t="s">
+      <c r="W21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="T21" s="5" t="s">
+      <c r="X21" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="U21" s="5" t="s">
+      <c r="Y21" s="5" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I22" s="2" t="s">
-        <v>150</v>
+    <row r="22" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I22" s="7">
+        <v>3</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>151</v>
@@ -2582,36 +2878,52 @@
       <c r="O22" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="Q22" s="4" t="s">
+      <c r="P22" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q22" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="S22" s="2">
+        <v>1</v>
+      </c>
+      <c r="U22" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="R22" s="4" t="s">
+      <c r="V22" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="S22" s="5" t="s">
+      <c r="W22" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="T22" s="5" t="s">
+      <c r="X22" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="U22" s="5" t="s">
+      <c r="Y22" s="5" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="24" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="I24" s="18" t="s">
+    <row r="24" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="I24" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="J24" s="18"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="18"/>
-      <c r="N24" s="18"/>
-      <c r="O24" s="18"/>
-    </row>
-    <row r="25" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
+      <c r="P24" s="13"/>
+      <c r="Q24" s="13"/>
+      <c r="R24" s="13"/>
+      <c r="S24" s="14"/>
+    </row>
+    <row r="25" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I25" s="1" t="s">
-        <v>36</v>
+        <v>291</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>0</v>
@@ -2631,10 +2943,22 @@
       <c r="O25" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="26" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I26" s="2" t="s">
-        <v>70</v>
+      <c r="P25" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q25" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="R25" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S25" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="26" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I26" s="7">
+        <v>1</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>100</v>
@@ -2654,25 +2978,37 @@
       <c r="O26" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q26" s="1" t="s">
+      <c r="P26" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="Q26" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="R26" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="S26" s="2">
+        <v>1</v>
+      </c>
+      <c r="U26" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="R26" s="1" t="s">
+      <c r="V26" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="S26" s="3" t="s">
+      <c r="W26" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="T26" s="3" t="s">
+      <c r="X26" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="U26" s="3" t="s">
+      <c r="Y26" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="27" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I27" s="2" t="s">
-        <v>71</v>
+    <row r="27" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I27" s="7">
+        <v>2</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>107</v>
@@ -2692,23 +3028,35 @@
       <c r="O27" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q27" s="1" t="s">
+      <c r="P27" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="Q27" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="R27" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S27" s="2">
+        <v>2</v>
+      </c>
+      <c r="U27" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="R27" s="1" t="s">
+      <c r="V27" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="S27" s="3" t="s">
+      <c r="W27" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="T27" s="3" t="s">
+      <c r="X27" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="U27" s="3" t="s">
+      <c r="Y27" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="29" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="29" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
       <c r="I29" s="15" t="s">
         <v>121</v>
       </c>
@@ -2717,11 +3065,15 @@
       <c r="L29" s="16"/>
       <c r="M29" s="16"/>
       <c r="N29" s="16"/>
-      <c r="O29" s="17"/>
-    </row>
-    <row r="30" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="O29" s="16"/>
+      <c r="P29" s="16"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="16"/>
+      <c r="S29" s="17"/>
+    </row>
+    <row r="30" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I30" s="4" t="s">
-        <v>36</v>
+        <v>291</v>
       </c>
       <c r="J30" s="4" t="s">
         <v>0</v>
@@ -2741,10 +3093,22 @@
       <c r="O30" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="31" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I31" s="2" t="s">
-        <v>70</v>
+      <c r="P30" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q30" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="R30" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="S30" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="31" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I31" s="7">
+        <v>1</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>111</v>
@@ -2764,25 +3128,37 @@
       <c r="O31" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q31" s="4" t="s">
+      <c r="P31" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="Q31" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="R31" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="S31" s="2">
+        <v>1</v>
+      </c>
+      <c r="U31" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="R31" s="4" t="s">
+      <c r="V31" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="S31" s="5" t="s">
+      <c r="W31" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="T31" s="5" t="s">
+      <c r="X31" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="U31" s="5" t="s">
+      <c r="Y31" s="5" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="32" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I32" s="2" t="s">
-        <v>71</v>
+    <row r="32" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I32" s="7">
+        <v>2</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>117</v>
@@ -2802,23 +3178,35 @@
       <c r="O32" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q32" s="4" t="s">
+      <c r="P32" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="Q32" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="R32" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="S32" s="2">
+        <v>2</v>
+      </c>
+      <c r="U32" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="R32" s="4" t="s">
+      <c r="V32" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="S32" s="5" t="s">
+      <c r="W32" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="T32" s="5" t="s">
+      <c r="X32" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="U32" s="5" t="s">
+      <c r="Y32" s="5" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="34" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="34" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
       <c r="I34" s="12" t="s">
         <v>132</v>
       </c>
@@ -2827,11 +3215,15 @@
       <c r="L34" s="13"/>
       <c r="M34" s="13"/>
       <c r="N34" s="13"/>
-      <c r="O34" s="14"/>
-    </row>
-    <row r="35" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="O34" s="13"/>
+      <c r="P34" s="13"/>
+      <c r="Q34" s="13"/>
+      <c r="R34" s="13"/>
+      <c r="S34" s="14"/>
+    </row>
+    <row r="35" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I35" s="1" t="s">
-        <v>36</v>
+        <v>291</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>0</v>
@@ -2851,10 +3243,22 @@
       <c r="O35" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="36" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I36" s="2" t="s">
-        <v>70</v>
+      <c r="P35" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q35" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="R35" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S35" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="36" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I36" s="7">
+        <v>1</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>125</v>
@@ -2874,25 +3278,37 @@
       <c r="O36" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="Q36" s="1" t="s">
+      <c r="P36" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="Q36" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="R36" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="S36" s="2">
+        <v>1</v>
+      </c>
+      <c r="U36" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="R36" s="1" t="s">
+      <c r="V36" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="S36" s="3" t="s">
+      <c r="W36" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="T36" s="3" t="s">
+      <c r="X36" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="U36" s="3" t="s">
+      <c r="Y36" s="3" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I37" s="2" t="s">
-        <v>157</v>
+    <row r="37" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I37" s="7">
+        <v>2</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>158</v>
@@ -2912,23 +3328,35 @@
       <c r="O37" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="Q37" s="1" t="s">
+      <c r="P37" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="Q37" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="R37" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="S37" s="2">
+        <v>2</v>
+      </c>
+      <c r="U37" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="R37" s="1" t="s">
+      <c r="V37" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="S37" s="3" t="s">
+      <c r="W37" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="T37" s="3" t="s">
+      <c r="X37" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="U37" s="3" t="s">
+      <c r="Y37" s="3" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="39" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="39" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
       <c r="I39" s="15" t="s">
         <v>133</v>
       </c>
@@ -2937,11 +3365,15 @@
       <c r="L39" s="16"/>
       <c r="M39" s="16"/>
       <c r="N39" s="16"/>
-      <c r="O39" s="17"/>
-    </row>
-    <row r="40" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="O39" s="16"/>
+      <c r="P39" s="16"/>
+      <c r="Q39" s="16"/>
+      <c r="R39" s="16"/>
+      <c r="S39" s="17"/>
+    </row>
+    <row r="40" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I40" s="4" t="s">
-        <v>36</v>
+        <v>291</v>
       </c>
       <c r="J40" s="4" t="s">
         <v>0</v>
@@ -2961,10 +3393,22 @@
       <c r="O40" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="41" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I41" s="2" t="s">
-        <v>70</v>
+      <c r="P40" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q40" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="R40" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="S40" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="41" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I41" s="7">
+        <v>1</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>135</v>
@@ -2984,25 +3428,37 @@
       <c r="O41" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Q41" s="4" t="s">
+      <c r="P41" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="Q41" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="R41" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="S41" s="2">
+        <v>1</v>
+      </c>
+      <c r="U41" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="R41" s="4" t="s">
+      <c r="V41" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="S41" s="5" t="s">
+      <c r="W41" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="T41" s="5" t="s">
+      <c r="X41" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="U41" s="5" t="s">
+      <c r="Y41" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="42" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I42" s="2" t="s">
-        <v>84</v>
+    <row r="42" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I42" s="7">
+        <v>2</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>139</v>
@@ -3022,25 +3478,37 @@
       <c r="O42" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q42" s="4" t="s">
+      <c r="P42" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="Q42" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="R42" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="S42" s="2">
+        <v>2</v>
+      </c>
+      <c r="U42" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="R42" s="4" t="s">
+      <c r="V42" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="S42" s="5" t="s">
+      <c r="W42" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="T42" s="5" t="s">
+      <c r="X42" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="U42" s="5" t="s">
+      <c r="Y42" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I43" s="2" t="s">
-        <v>134</v>
+    <row r="43" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I43" s="7">
+        <v>3</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>143</v>
@@ -3060,23 +3528,35 @@
       <c r="O43" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q43" s="4" t="s">
+      <c r="P43" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="Q43" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="R43" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="S43" s="2">
+        <v>1</v>
+      </c>
+      <c r="U43" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="R43" s="4" t="s">
+      <c r="V43" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="S43" s="5" t="s">
+      <c r="W43" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="T43" s="5" t="s">
+      <c r="X43" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="U43" s="5" t="s">
+      <c r="Y43" s="5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="46" spans="9:21" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="46" spans="9:25" ht="18.75" x14ac:dyDescent="0.3">
       <c r="I46" s="11" t="s">
         <v>170</v>
       </c>
@@ -3086,10 +3566,14 @@
       <c r="M46" s="11"/>
       <c r="N46" s="11"/>
       <c r="O46" s="11"/>
-    </row>
-    <row r="47" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="P46" s="11"/>
+      <c r="Q46" s="11"/>
+      <c r="R46" s="11"/>
+      <c r="S46" s="11"/>
+    </row>
+    <row r="47" spans="9:25" x14ac:dyDescent="0.25">
       <c r="I47" s="6" t="s">
-        <v>199</v>
+        <v>291</v>
       </c>
       <c r="J47" s="6" t="s">
         <v>0</v>
@@ -3109,10 +3593,22 @@
       <c r="O47" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="48" spans="9:21" x14ac:dyDescent="0.25">
-      <c r="I48" s="7" t="s">
-        <v>200</v>
+      <c r="P47" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q47" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="R47" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="S47" s="6" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="48" spans="9:25" x14ac:dyDescent="0.25">
+      <c r="I48" s="7">
+        <v>1</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>192</v>
@@ -3132,10 +3628,23 @@
       <c r="O48" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="49" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I49" s="7" t="s">
-        <v>201</v>
+      <c r="P48" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q48" s="2" t="str">
+        <f>K48 &amp; " - " &amp; L48</f>
+        <v>183.168.100.1 - 183.168.100.2</v>
+      </c>
+      <c r="R48" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="S48" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I49" s="7">
+        <v>2</v>
       </c>
       <c r="J49" s="2" t="s">
         <v>193</v>
@@ -3155,10 +3664,23 @@
       <c r="O49" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="50" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I50" s="7" t="s">
-        <v>202</v>
+      <c r="P49" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q49" s="2" t="str">
+        <f t="shared" ref="Q49:Q55" si="0">K49 &amp; " - " &amp; L49</f>
+        <v>183.168.100.5 - 183.168.100.6</v>
+      </c>
+      <c r="R49" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="S49" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I50" s="7">
+        <v>3</v>
       </c>
       <c r="J50" s="2" t="s">
         <v>194</v>
@@ -3178,10 +3700,23 @@
       <c r="O50" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="51" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I51" s="7" t="s">
-        <v>203</v>
+      <c r="P50" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q50" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>183.168.100.9 - 183.168.100.10</v>
+      </c>
+      <c r="R50" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="S50" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I51" s="7">
+        <v>4</v>
       </c>
       <c r="J51" s="2" t="s">
         <v>195</v>
@@ -3201,10 +3736,23 @@
       <c r="O51" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="52" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I52" s="7" t="s">
-        <v>204</v>
+      <c r="P51" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q51" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>183.168.100.13 - 183.168.100.14</v>
+      </c>
+      <c r="R51" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="S51" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I52" s="7">
+        <v>5</v>
       </c>
       <c r="J52" s="2" t="s">
         <v>196</v>
@@ -3224,10 +3772,23 @@
       <c r="O52" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="53" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I53" s="7" t="s">
-        <v>205</v>
+      <c r="P52" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q52" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>183.168.100.17 - 183.168.100.18</v>
+      </c>
+      <c r="R52" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="S52" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I53" s="7">
+        <v>6</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>198</v>
@@ -3247,10 +3808,23 @@
       <c r="O53" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="54" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I54" s="7" t="s">
-        <v>206</v>
+      <c r="P53" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q53" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>183.168.100.21 - 183.168.100.22</v>
+      </c>
+      <c r="R53" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="S53" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I54" s="7">
+        <v>7</v>
       </c>
       <c r="J54" s="2" t="s">
         <v>197</v>
@@ -3270,22 +3844,35 @@
       <c r="O54" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="55" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I55" s="7" t="s">
-        <v>207</v>
+      <c r="P54" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q54" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>183.168.100.25 - 183.168.100.26</v>
+      </c>
+      <c r="R54" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="S54" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I55" s="7">
+        <v>8</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="N55" s="2" t="s">
         <v>156</v>
@@ -3293,169 +3880,168 @@
       <c r="O55" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="56" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I56" s="20" t="s">
-        <v>254</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="N56" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="O56" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="58" spans="9:15" x14ac:dyDescent="0.25">
+      <c r="P55" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q55" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>183.168.100.29 - 183.168.100.30</v>
+      </c>
+      <c r="R55" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="S55" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I56" s="20"/>
+      <c r="J56" s="19"/>
+      <c r="K56" s="19"/>
+      <c r="L56" s="19"/>
+      <c r="M56" s="19"/>
+      <c r="N56" s="19"/>
+      <c r="O56" s="19"/>
+    </row>
+    <row r="58" spans="9:19" x14ac:dyDescent="0.25">
       <c r="I58" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="J58" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="K58" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="L58" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="M58" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="N58" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="O58" s="10" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="59" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I59" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="J59" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="K59" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="L59" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="M59" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="N59" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="O59" s="10" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="60" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I60" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="J60" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="K60" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="L60" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="M60" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="N60" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="O60" s="10" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="61" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I61" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="J61" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="K61" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="L61" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="M61" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="N61" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="O61" s="10" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="62" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I62" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="J62" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="J58" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="K58" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="L58" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="M58" s="10" t="s">
+      <c r="K62" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="L62" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="N58" s="10" t="s">
-        <v>242</v>
-      </c>
-      <c r="O58" s="10" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="59" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I59" s="9" t="s">
+      <c r="M62" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="N62" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="O62" s="10" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="63" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I63" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="J63" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="J59" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="K59" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="L59" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="M59" s="10" t="s">
+      <c r="K63" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="L63" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="N59" s="10" t="s">
-        <v>243</v>
-      </c>
-      <c r="O59" s="10" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="60" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I60" s="9" t="s">
-        <v>215</v>
-      </c>
-      <c r="J60" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="K60" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="L60" s="10" t="s">
+      <c r="M63" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="N63" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="M60" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="N60" s="10" t="s">
+      <c r="O63" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="O60" s="10" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="61" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I61" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="J61" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="K61" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="L61" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="M61" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="N61" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="O61" s="10" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="62" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I62" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="J62" s="10" t="s">
-        <v>222</v>
-      </c>
-      <c r="K62" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="L62" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="M62" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="N62" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="O62" s="10" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="63" spans="9:15" x14ac:dyDescent="0.25">
-      <c r="I63" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="J63" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="K63" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="L63" s="10" t="s">
-        <v>241</v>
-      </c>
-      <c r="M63" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="N63" s="10" t="s">
-        <v>247</v>
-      </c>
-      <c r="O63" s="10" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="64" spans="9:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="9:19" x14ac:dyDescent="0.25">
       <c r="I64" s="8"/>
     </row>
     <row r="65" spans="9:9" x14ac:dyDescent="0.25">
@@ -3466,15 +4052,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="I46:O46"/>
-    <mergeCell ref="I34:O34"/>
-    <mergeCell ref="I39:O39"/>
-    <mergeCell ref="I29:O29"/>
-    <mergeCell ref="I1:O1"/>
-    <mergeCell ref="I7:O7"/>
-    <mergeCell ref="I13:O13"/>
-    <mergeCell ref="I18:O18"/>
-    <mergeCell ref="I24:O24"/>
+    <mergeCell ref="I39:S39"/>
+    <mergeCell ref="I46:S46"/>
+    <mergeCell ref="I1:S1"/>
+    <mergeCell ref="I7:S7"/>
+    <mergeCell ref="I13:S13"/>
+    <mergeCell ref="I18:S18"/>
+    <mergeCell ref="I24:S24"/>
+    <mergeCell ref="I29:S29"/>
+    <mergeCell ref="I34:S34"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>